<commit_message>
Preserve typed custom arguments and failed lookup source expressions
</commit_message>
<xml_diff>
--- a/OfficeIMO.TestAssets/Documents/ExcelFormulaCorpus/lookup-conformance-windows.xlsx
+++ b/OfficeIMO.TestAssets/Documents/ExcelFormulaCorpus/lookup-conformance-windows.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Support\GitHub\_worktrees\OfficeIMO-formula-errors\OfficeIMO.TestAssets\Documents\ExcelFormulaCorpus\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1059DBE3-3FBC-423F-B9E5-77BB31BB8D28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA9E8511-7492-40BD-B704-A79E934E5AE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -943,7 +943,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D1701"/>
+  <dimension ref="A1:D1811"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
@@ -2371,6 +2371,72 @@
       </c>
       <c r="B1701" t="str">
         <v>E</v>
+      </c>
+    </row>
+    <row r="1711" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1711" t="e">
+        <f>MATCH(1,1/0,0)</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="1721" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1721" t="e">
+        <f>_xlfn.XMATCH(1,1/0)</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="1731" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1731" t="e">
+        <f>VLOOKUP(1,1/0,1,FALSE)</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="1741" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1741" t="e">
+        <f>HLOOKUP(1,1/0,1,FALSE)</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="1751" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1751" t="e" cm="1">
+        <f t="array" ref="A1751">_xlfn.XLOOKUP(1,1/0,{10})</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="1761" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1761" t="e">
+        <f>_xlfn.IFNA(MATCH(1,1/0,0),99)</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="1771" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1771" t="e">
+        <f>MATCH(1,{#DIV/0!},0)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="1781" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1781" t="e">
+        <f>_xlfn.XMATCH(1,{#DIV/0!})</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="1791" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1791" t="e">
+        <f>VLOOKUP(1,{#DIV/0!},1,FALSE)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="1801" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1801" t="e">
+        <f>HLOOKUP(1,{#DIV/0!},1,FALSE)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="1811" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1811" t="e" cm="1">
+        <f t="array" ref="A1811">_xlfn.XLOOKUP(1,{#DIV/0!},{10})</f>
+        <v>#N/A</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Calculate SUMPRODUCT blank and mixed-type inputs using native semantics
</commit_message>
<xml_diff>
--- a/OfficeIMO.TestAssets/Documents/ExcelFormulaCorpus/lookup-conformance-windows.xlsx
+++ b/OfficeIMO.TestAssets/Documents/ExcelFormulaCorpus/lookup-conformance-windows.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Support\GitHub\_worktrees\OfficeIMO-formula-errors\OfficeIMO.TestAssets\Documents\ExcelFormulaCorpus\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA9E8511-7492-40BD-B704-A79E934E5AE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1C77A5A-C924-4E51-891E-863910EAABFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -943,7 +943,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D1811"/>
+  <dimension ref="A1:D2071"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
@@ -2436,6 +2436,168 @@
     <row r="1811" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1811" t="e" cm="1">
         <f t="array" ref="A1811">_xlfn.XLOOKUP(1,{#DIV/0!},{10})</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="1821" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1821">
+        <f>SUMPRODUCT(Data!A1:A5,Data!F1:F5)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="1831" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1831">
+        <f>SUMPRODUCT(Data!F1:F5)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1841" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1841">
+        <f>SUMPRODUCT(Data!A1:A5,Data!F1:F5,Data!F1:F5)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="1851" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1851" t="e">
+        <f>SUMPRODUCT(Data!F5,2)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="1861" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1861" t="e">
+        <f>SUMPRODUCT(INDEX(Data!F1:F6,5),2)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="1871" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1871" t="e">
+        <f>SUMPRODUCT(IFERROR(Data!F5,77),2)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="1881" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1881">
+        <f>SUMPRODUCT(TRUE,2)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1891" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1891">
+        <f>SUMPRODUCT("1",2)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1901" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1901">
+        <f>SUMPRODUCT({1;"1";TRUE;FALSE;0},{10;20;30;40;50})</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="1911" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1911" t="e">
+        <f>SUMPRODUCT(Data!F5,NA())</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="1921" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1921" t="e">
+        <f>SUMPRODUCT(Data!F1:F6,Data!A1:A6)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="1931" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1931">
+        <f>IFERROR(SUMPRODUCT(Data!F1:F5,Data!A1:A5),99)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="1941" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1941" cm="1">
+        <f t="array" ref="A1941:B1941">INDEX({10,20;30,40},2)</f>
+        <v>30</v>
+      </c>
+      <c r="B1941">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="1951" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1951">
+        <f>SUM(INDEX({10,20;30,40},2))</f>
+        <v>70</v>
+      </c>
+    </row>
+    <row r="1961" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1961" cm="1">
+        <f t="array" ref="A1961:B1961">INDEX({10,20;30,40},2,)</f>
+        <v>30</v>
+      </c>
+      <c r="B1961">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="1971" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1971" t="e">
+        <f>SUMPRODUCT(Data!F5,Data!F5)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="1981" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1981" t="e">
+        <f>SUMPRODUCT(Data!F5)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="1991" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1991" t="e">
+        <f>SUMPRODUCT(Data!F5:F5,{2})</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="2001" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2001">
+        <f>SUMPRODUCT(0,2)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2011" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2011">
+        <f>SUMPRODUCT(Data!F2,2)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2021" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2021">
+        <f>SUMPRODUCT(Data!F3,2)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2031" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2031" t="e">
+        <f>SUMPRODUCT(NA(),Data!F5)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="2041" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2041" t="e">
+        <f>SUMPRODUCT({#N/A;0},{0;0})</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="2051" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2051">
+        <f>SUMPRODUCT({"";0},{2;3})</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2061" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2061">
+        <f>SUMPRODUCT(Data!F4:F5,Data!A1:A2)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2071" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2071" t="e">
+        <f>SUMPRODUCT(Data!F5:F6,Data!A1:A2)</f>
         <v>#N/A</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Validate SUMPRODUCT array dimensions before publishing results
</commit_message>
<xml_diff>
--- a/OfficeIMO.TestAssets/Documents/ExcelFormulaCorpus/lookup-conformance-windows.xlsx
+++ b/OfficeIMO.TestAssets/Documents/ExcelFormulaCorpus/lookup-conformance-windows.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Support\GitHub\_worktrees\OfficeIMO-formula-errors\OfficeIMO.TestAssets\Documents\ExcelFormulaCorpus\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1C77A5A-C924-4E51-891E-863910EAABFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E32F1F4-48AF-4B7A-AA9D-DEDAF7595D1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -943,7 +943,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D2071"/>
+  <dimension ref="A1:D2171"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
@@ -2598,6 +2598,66 @@
     <row r="2071" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2071" t="e">
         <f>SUMPRODUCT(Data!F5:F6,Data!A1:A2)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="2081" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2081" t="e">
+        <f>SUMPRODUCT({1,2},{3;4})</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="2091" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2091" t="e">
+        <f>SUMPRODUCT({1,2;3,4},{5;6;7;8})</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="2101" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2101">
+        <f>SUMPRODUCT({1,2;3,4},{5,6;7,8})</f>
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2111" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2111" t="e">
+        <f>SUMPRODUCT({1;2},{3;4;5})</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="2121" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2121" t="e">
+        <f>SUMPRODUCT(2,{3;4})</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="2131" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2131" t="e">
+        <f>SUMPRODUCT(NA(),{3;4})</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="2141" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2141" t="e">
+        <f>SUMPRODUCT({1;2},{#N/A;2;3})</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="2151" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2151" t="e">
+        <f>SUMPRODUCT({#N/A;2},{1;2;3})</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="2161" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2161" t="e">
+        <f>SUMPRODUCT({#N/A},{1;2})</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="2171" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2171" t="e">
+        <f>SUMPRODUCT(Data!F6,{1;2})</f>
         <v>#N/A</v>
       </c>
     </row>

</xml_diff>